<commit_message>
🔄 Mise à jour du fichier Excel public
</commit_message>
<xml_diff>
--- a/docs/epexspot_prices.xlsx
+++ b/docs/epexspot_prices.xlsx
@@ -17162,7 +17162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B253"/>
+  <dimension ref="A1:B254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19689,6 +19689,16 @@
       </c>
       <c r="B253" t="n">
         <v>30.5</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>42.1</v>
       </c>
     </row>
   </sheetData>
@@ -19702,7 +19712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B249"/>
+  <dimension ref="A1:B250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22167,6 +22177,16 @@
         <v>70.43000000000001</v>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>